<commit_message>
Start dev of excel module
</commit_message>
<xml_diff>
--- a/data/regime.xlsx
+++ b/data/regime.xlsx
@@ -24,10 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
-  <si>
-    <t/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Calories</t>
   </si>
@@ -64,7 +61,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -75,6 +72,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -97,7 +100,14 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -126,47 +136,47 @@
   </cellStyleXfs>
   <cellXfs count="15">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -473,188 +483,184 @@
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="12" width="11.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="11.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="13" width="11.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="11.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="11.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="11" width="11.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="13.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="13" width="13.005" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="13" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="12" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="13.005" customWidth="1" bestFit="1"/>
     <col min="8" max="8" style="13" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="3"/>
+      <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="4"/>
+      <c r="G1" s="3"/>
       <c r="H1" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
-      <c r="A2" s="4"/>
+      <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="3"/>
+      <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="4"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
-      <c r="A3" s="5"/>
-      <c r="B3" s="6" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="4"/>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="3"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="4"/>
-      <c r="H3" s="7" t="s">
+      <c r="B4" s="7">
+        <v>400</v>
+      </c>
+      <c r="C4" s="7">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7">
+        <v>2</v>
+      </c>
+      <c r="E4" s="7">
+        <v>2</v>
+      </c>
+      <c r="F4" s="7">
+        <v>50</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="7">
+        <v>200</v>
+      </c>
+      <c r="C5" s="7">
+        <v>2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>2</v>
+      </c>
+      <c r="E5" s="7">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7">
+        <v>20</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="7">
+        <v>150</v>
+      </c>
+      <c r="C6" s="7">
         <v>0</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
-      <c r="A4" s="5" t="s">
+      <c r="D6" s="7">
+        <v>4</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7">
+        <v>30</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="7">
+        <v>500</v>
+      </c>
+      <c r="C7" s="7">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7">
+        <v>4</v>
+      </c>
+      <c r="E7" s="7">
+        <v>5</v>
+      </c>
+      <c r="F7" s="7">
+        <v>80</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7">
+        <v>500</v>
+      </c>
+      <c r="C8" s="7">
         <v>6</v>
       </c>
-      <c r="B4" s="8">
-        <v>400</v>
-      </c>
-      <c r="C4" s="8">
-        <v>3</v>
-      </c>
-      <c r="D4" s="8">
-        <v>2</v>
-      </c>
-      <c r="E4" s="8">
-        <v>2</v>
-      </c>
-      <c r="F4" s="8">
-        <v>50</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
-      <c r="A5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="8">
-        <v>200</v>
-      </c>
-      <c r="C5" s="8">
-        <v>2</v>
-      </c>
-      <c r="D5" s="8">
-        <v>2</v>
-      </c>
-      <c r="E5" s="8">
-        <v>4</v>
-      </c>
-      <c r="F5" s="8">
-        <v>20</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
-      <c r="A6" s="5" t="s">
+      <c r="D8" s="7">
+        <v>10</v>
+      </c>
+      <c r="E8" s="7">
         <v>8</v>
       </c>
-      <c r="B6" s="8">
-        <v>150</v>
-      </c>
-      <c r="C6" s="8">
-        <v>0</v>
-      </c>
-      <c r="D6" s="8">
-        <v>4</v>
-      </c>
-      <c r="E6" s="8">
-        <v>1</v>
-      </c>
-      <c r="F6" s="8">
-        <v>30</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="8">
-        <v>500</v>
-      </c>
-      <c r="C7" s="8">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
-        <v>4</v>
-      </c>
-      <c r="E7" s="8">
-        <v>5</v>
-      </c>
-      <c r="F7" s="8">
-        <v>80</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="9"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="8">
-        <v>500</v>
-      </c>
-      <c r="C8" s="8">
-        <v>6</v>
-      </c>
-      <c r="D8" s="8">
-        <v>10</v>
-      </c>
-      <c r="E8" s="8">
-        <v>8</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="4"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="3"/>
       <c r="H8" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
-      <c r="A9" s="4"/>
+      <c r="A9" s="1"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
-      <c r="G9" s="4"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="11"/>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+      <c r="A10" s="4"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="9">
+        <v>90</v>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
-      <c r="G10" s="4"/>
+      <c r="G10" s="3"/>
       <c r="H10" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cleaning module general upgrades
</commit_message>
<xml_diff>
--- a/data/regime.xlsx
+++ b/data/regime.xlsx
@@ -134,46 +134,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -487,13 +484,13 @@
     <col min="2" max="2" style="11" width="11.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="11" width="11.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="12" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="13" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="13" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="13" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="13" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -503,7 +500,7 @@
       <c r="G1" s="3"/>
       <c r="H1" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -641,7 +638,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -655,9 +652,7 @@
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="9">
-        <v>90</v>
-      </c>
+      <c r="D10" s="9"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10" s="3"/>

</xml_diff>